<commit_message>
Complete homepage redesign - clean professional layout
</commit_message>
<xml_diff>
--- a/total Tools.xlsx
+++ b/total Tools.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Shailesh\PrimeTools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AEBBB695-84EB-4B8E-A8A0-5A712B5C814E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30F37007-EAF6-43B7-9051-A484A8DF0FF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{53663192-2907-4C22-A177-13377D2CEE9C}"/>
   </bookViews>
@@ -243,7 +243,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -251,15 +251,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -598,8 +614,8 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -618,632 +634,632 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6">
+      <c r="A6" s="2">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8">
+      <c r="A8" s="2">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9">
+      <c r="A9" s="2">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10">
+      <c r="A10" s="2">
         <v>9</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11">
+      <c r="A11" s="2">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12">
+      <c r="A12" s="2">
         <v>11</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13">
+      <c r="A13" s="2">
         <v>12</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14">
+      <c r="A14" s="2">
         <v>13</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15">
+      <c r="A15" s="2">
         <v>14</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16">
+      <c r="A16" s="2">
         <v>15</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17">
+      <c r="A17" s="2">
         <v>16</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18">
+      <c r="A18" s="2">
         <v>17</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19">
+      <c r="A19" s="2">
         <v>18</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20">
+      <c r="A20" s="2">
         <v>19</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21">
+      <c r="A21" s="2">
         <v>20</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22">
+      <c r="A22" s="2">
         <v>21</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23">
+      <c r="A23" s="2">
         <v>22</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24">
+      <c r="A24" s="2">
         <v>23</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25">
+      <c r="A25" s="2">
         <v>24</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26">
+      <c r="A26" s="2">
         <v>25</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27">
+      <c r="A27" s="2">
         <v>26</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28">
+      <c r="A28" s="2">
         <v>27</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D28" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29">
+      <c r="A29" s="2">
         <v>28</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D29" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30">
+      <c r="A30" s="2">
         <v>29</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31">
+      <c r="A31" s="2">
         <v>30</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D31" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32">
+      <c r="A32" s="2">
         <v>31</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D32" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33">
+      <c r="A33" s="2">
         <v>32</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C33" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D33" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34">
+      <c r="A34" s="2">
         <v>33</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C34" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D34" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35">
+      <c r="A35" s="2">
         <v>34</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C35" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D35" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A36">
+      <c r="A36" s="2">
         <v>35</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C36" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D36" t="s">
+      <c r="D36" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A37">
+      <c r="A37" s="2">
         <v>36</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C37" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D37" t="s">
+      <c r="D37" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A38">
+      <c r="A38" s="2">
         <v>37</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C38" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D38" t="s">
+      <c r="D38" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A39">
+      <c r="A39" s="2">
         <v>38</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C39" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D39" t="s">
+      <c r="D39" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A40">
+      <c r="A40" s="2">
         <v>39</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B40" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C40" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D40" t="s">
+      <c r="D40" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A41">
+      <c r="A41" s="2">
         <v>40</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B41" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C41" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D41" t="s">
+      <c r="D41" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A42">
+      <c r="A42" s="2">
         <v>41</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B42" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C42" t="s">
+      <c r="C42" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D42" t="s">
+      <c r="D42" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A43">
+      <c r="A43" s="2">
         <v>42</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B43" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C43" t="s">
+      <c r="C43" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="D43" t="s">
+      <c r="D43" s="2" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A44">
+      <c r="A44" s="2">
         <v>43</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C44" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="D44" t="s">
+      <c r="D44" s="2" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A45">
+      <c r="A45" s="2">
         <v>44</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B45" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C45" t="s">
+      <c r="C45" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="D45" t="s">
+      <c r="D45" s="2" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A46">
+      <c r="A46" s="2">
         <v>45</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B46" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C46" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="D46" t="s">
+      <c r="D46" s="2" t="s">
         <v>55</v>
       </c>
     </row>

</xml_diff>